<commit_message>
Actualizacion dashboard con consultor JBL
</commit_message>
<xml_diff>
--- a/IXComercio.xlsx
+++ b/IXComercio.xlsx
@@ -426,7 +426,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E16"/>
+  <dimension ref="A1:E17"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -836,6 +836,31 @@
         <v>965</v>
       </c>
     </row>
+    <row r="17">
+      <c r="A17" t="inlineStr">
+        <is>
+          <t>17/09/2026</t>
+        </is>
+      </c>
+      <c r="B17" t="inlineStr">
+        <is>
+          <t>Total ordenes IX</t>
+        </is>
+      </c>
+      <c r="C17" t="inlineStr">
+        <is>
+          <t>Todos</t>
+        </is>
+      </c>
+      <c r="D17" t="inlineStr">
+        <is>
+          <t>Web</t>
+        </is>
+      </c>
+      <c r="E17" t="n">
+        <v>840</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>